<commit_message>
Flight crew scheduling: review fixes
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/flightcrewscheduling/unsolved/175flights-7days-Europe.xlsx
+++ b/optaplanner-examples/data/flightcrewscheduling/unsolved/175flights-7days-Europe.xlsx
@@ -6724,10 +6724,10 @@
       <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F3" s="3" t="s">
@@ -6855,7 +6855,7 @@
       <c r="D7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -6864,10 +6864,10 @@
       <c r="G7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="H7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J7" s="2" t="s">
@@ -6980,7 +6980,7 @@
       <c r="C11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -6989,10 +6989,10 @@
       <c r="F11" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H11" s="3" t="s">
+      <c r="G11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -7007,7 +7007,7 @@
         <v>92</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>18</v>
@@ -7027,7 +7027,7 @@
       <c r="H12" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="3" t="s">
         <v>74</v>
       </c>
       <c r="J12" s="2" t="s">
@@ -7044,7 +7044,7 @@
       <c r="C13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -7056,13 +7056,13 @@
       <c r="G13" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J13" s="3" t="s">
+      <c r="H13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -7079,16 +7079,16 @@
       <c r="D14" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="E14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="3" t="s">
         <v>74</v>
       </c>
       <c r="I14" s="2" t="s">
@@ -7239,13 +7239,13 @@
       <c r="D19" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G19" s="3" t="s">
+      <c r="E19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H19" s="2" t="s">
@@ -7271,10 +7271,10 @@
       <c r="D20" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F20" s="3" t="s">
+      <c r="E20" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G20" s="2" t="s">
@@ -7286,7 +7286,7 @@
       <c r="I20" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J20" s="3" t="s">
+      <c r="J20" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
         <v>101</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>18</v>
@@ -7315,10 +7315,10 @@
       <c r="H21" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J21" s="2" t="s">
+      <c r="I21" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -7359,7 +7359,7 @@
         <v>103</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
@@ -7437,16 +7437,16 @@
       <c r="F25" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="J25" s="3" t="s">
+      <c r="G25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       <c r="C26" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E26" s="2" t="s">
@@ -7469,7 +7469,7 @@
       <c r="F26" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H26" s="2" t="s">
@@ -7487,7 +7487,7 @@
         <v>107</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>18</v>
@@ -7519,7 +7519,7 @@
         <v>108</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>17</v>
@@ -7647,7 +7647,7 @@
         <v>112</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>18</v>
@@ -7655,10 +7655,10 @@
       <c r="D32" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F32" s="3" t="s">
+      <c r="E32" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G32" s="2" t="s">
@@ -7679,7 +7679,7 @@
         <v>113</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>17</v>
@@ -7696,10 +7696,10 @@
       <c r="G33" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H33" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I33" s="3" t="s">
+      <c r="H33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J33" s="2" t="s">
@@ -7711,7 +7711,7 @@
         <v>114</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>17</v>
@@ -7748,7 +7748,7 @@
       <c r="C35" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -7766,7 +7766,7 @@
       <c r="I35" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J35" s="3" t="s">
+      <c r="J35" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
         <v>116</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>18</v>
@@ -7789,7 +7789,7 @@
       <c r="F36" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="3" t="s">
         <v>74</v>
       </c>
       <c r="H36" s="2" t="s">
@@ -7847,7 +7847,7 @@
       <c r="D38" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F38" s="2" t="s">
@@ -7856,7 +7856,7 @@
       <c r="G38" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I38" s="2" t="s">
@@ -7871,7 +7871,7 @@
         <v>119</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>17</v>
@@ -7903,7 +7903,7 @@
         <v>120</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>18</v>
@@ -7935,7 +7935,7 @@
         <v>121</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>18</v>
@@ -7955,7 +7955,7 @@
       <c r="H41" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="I41" s="3" t="s">
         <v>74</v>
       </c>
       <c r="J41" s="2" t="s">
@@ -7999,7 +7999,7 @@
         <v>123</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>17</v>
@@ -8010,16 +8010,16 @@
       <c r="E43" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H43" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I43" s="3" t="s">
+      <c r="H43" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J43" s="2" t="s">
@@ -8031,7 +8031,7 @@
         <v>124</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>17</v>
@@ -8063,27 +8063,27 @@
         <v>125</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="D45" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F45" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G45" s="3" t="s">
+      <c r="F45" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I45" s="3" t="s">
+      <c r="I45" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J45" s="2" t="s">
@@ -8095,7 +8095,7 @@
         <v>126</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>18</v>
@@ -8127,7 +8127,7 @@
         <v>127</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>18</v>
@@ -8135,7 +8135,7 @@
       <c r="D47" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F47" s="2" t="s">
@@ -8150,7 +8150,7 @@
       <c r="I47" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J47" s="3" t="s">
+      <c r="J47" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8159,7 +8159,7 @@
         <v>128</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>17</v>
@@ -8191,7 +8191,7 @@
         <v>129</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>17</v>
@@ -8223,7 +8223,7 @@
         <v>130</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>18</v>
@@ -8287,24 +8287,24 @@
         <v>132</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D52" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F52" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H52" s="3" t="s">
+      <c r="H52" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I52" s="2" t="s">
@@ -8333,7 +8333,7 @@
       <c r="F53" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G53" s="3" t="s">
+      <c r="G53" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H53" s="2" t="s">
@@ -8351,7 +8351,7 @@
         <v>134</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>17</v>
@@ -8374,7 +8374,7 @@
       <c r="I54" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J54" s="2" t="s">
+      <c r="J54" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8388,25 +8388,25 @@
       <c r="C55" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F55" s="3" t="s">
+      <c r="D55" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H55" s="3" t="s">
+      <c r="H55" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J55" s="3" t="s">
+      <c r="J55" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8447,7 +8447,7 @@
         <v>137</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>18</v>
@@ -8502,7 +8502,7 @@
       <c r="I58" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J58" s="2" t="s">
+      <c r="J58" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
         <v>139</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>17</v>
@@ -8543,7 +8543,7 @@
         <v>140</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>18</v>
@@ -8607,7 +8607,7 @@
         <v>142</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>18</v>
@@ -8624,7 +8624,7 @@
       <c r="G62" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H62" s="2" t="s">
+      <c r="H62" s="3" t="s">
         <v>74</v>
       </c>
       <c r="I62" s="2" t="s">
@@ -8639,7 +8639,7 @@
         <v>143</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>17</v>
@@ -8653,13 +8653,13 @@
       <c r="F63" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G63" s="3" t="s">
+      <c r="G63" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I63" s="3" t="s">
+      <c r="I63" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J63" s="2" t="s">
@@ -8688,10 +8688,10 @@
       <c r="G64" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H64" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I64" s="3" t="s">
+      <c r="H64" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I64" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J64" s="2" t="s">
@@ -8708,7 +8708,7 @@
       <c r="C65" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D65" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E65" s="2" t="s">
@@ -8717,7 +8717,7 @@
       <c r="F65" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="G65" s="3" t="s">
         <v>74</v>
       </c>
       <c r="H65" s="2" t="s">
@@ -8735,7 +8735,7 @@
         <v>146</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>18</v>
@@ -8746,7 +8746,7 @@
       <c r="E66" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="F66" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G66" s="2" t="s">
@@ -8772,7 +8772,7 @@
       <c r="C67" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D67" s="3" t="s">
+      <c r="D67" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E67" s="2" t="s">
@@ -8790,7 +8790,7 @@
       <c r="I67" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J67" s="3" t="s">
+      <c r="J67" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8799,7 +8799,7 @@
         <v>148</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>17</v>
@@ -8839,10 +8839,10 @@
       <c r="D69" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E69" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F69" s="3" t="s">
+      <c r="E69" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F69" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G69" s="2" t="s">
@@ -8851,7 +8851,7 @@
       <c r="H69" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="I69" s="3" t="s">
         <v>74</v>
       </c>
       <c r="J69" s="2" t="s">
@@ -8863,7 +8863,7 @@
         <v>150</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>18</v>
@@ -8871,7 +8871,7 @@
       <c r="D70" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F70" s="2" t="s">
@@ -8886,7 +8886,7 @@
       <c r="I70" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J70" s="3" t="s">
+      <c r="J70" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -8900,22 +8900,22 @@
       <c r="C71" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D71" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E71" s="2" t="s">
+      <c r="D71" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E71" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G71" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I71" s="3" t="s">
+      <c r="G71" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I71" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J71" s="2" t="s">
@@ -8927,7 +8927,7 @@
         <v>152</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>18</v>
@@ -8959,30 +8959,30 @@
         <v>153</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D73" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E73" s="3" t="s">
+      <c r="D73" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F73" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G73" s="3" t="s">
+      <c r="G73" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I73" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J73" s="3" t="s">
+      <c r="I73" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J73" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9046,7 +9046,7 @@
       <c r="I75" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J75" s="2" t="s">
+      <c r="J75" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
         <v>156</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>18</v>
@@ -9066,13 +9066,13 @@
       <c r="E76" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F76" s="3" t="s">
+      <c r="F76" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H76" s="3" t="s">
+      <c r="H76" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I76" s="2" t="s">
@@ -9087,7 +9087,7 @@
         <v>157</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>18</v>
@@ -9119,12 +9119,12 @@
         <v>158</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="D78" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E78" s="2" t="s">
@@ -9151,7 +9151,7 @@
         <v>159</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>17</v>
@@ -9183,7 +9183,7 @@
         <v>160</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>18</v>
@@ -9215,7 +9215,7 @@
         <v>161</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>18</v>
@@ -9223,7 +9223,7 @@
       <c r="D81" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E81" s="3" t="s">
+      <c r="E81" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F81" s="2" t="s">
@@ -9235,7 +9235,7 @@
       <c r="H81" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I81" s="3" t="s">
+      <c r="I81" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J81" s="2" t="s">
@@ -9247,18 +9247,18 @@
         <v>162</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D82" s="3" t="s">
+      <c r="D82" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F82" s="3" t="s">
+      <c r="F82" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G82" s="2" t="s">
@@ -9279,7 +9279,7 @@
         <v>163</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
@@ -9302,7 +9302,7 @@
       <c r="I83" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J83" s="3" t="s">
+      <c r="J83" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9311,7 +9311,7 @@
         <v>164</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
@@ -9343,12 +9343,12 @@
         <v>165</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D85" s="3" t="s">
+      <c r="D85" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E85" s="2" t="s">
@@ -9389,7 +9389,7 @@
       <c r="F86" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G86" s="2" t="s">
+      <c r="G86" s="3" t="s">
         <v>74</v>
       </c>
       <c r="H86" s="2" t="s">
@@ -9430,7 +9430,7 @@
       <c r="I87" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J87" s="2" t="s">
+      <c r="J87" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9447,22 +9447,22 @@
       <c r="D88" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E88" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F88" s="3" t="s">
+      <c r="E88" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F88" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H88" s="3" t="s">
+      <c r="H88" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I88" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J88" s="3" t="s">
+      <c r="J88" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9503,7 +9503,7 @@
         <v>170</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>18</v>
@@ -9514,7 +9514,7 @@
       <c r="E90" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F90" s="2" t="s">
+      <c r="F90" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G90" s="2" t="s">
@@ -9540,13 +9540,13 @@
       <c r="C91" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D91" s="3" t="s">
+      <c r="D91" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F91" s="3" t="s">
+      <c r="F91" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G91" s="2" t="s">
@@ -9567,7 +9567,7 @@
         <v>172</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>18</v>
@@ -9575,7 +9575,7 @@
       <c r="D92" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E92" s="3" t="s">
+      <c r="E92" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F92" s="2" t="s">
@@ -9584,10 +9584,10 @@
       <c r="G92" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H92" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I92" s="2" t="s">
+      <c r="H92" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I92" s="3" t="s">
         <v>74</v>
       </c>
       <c r="J92" s="2" t="s">
@@ -9663,7 +9663,7 @@
         <v>175</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>18</v>
@@ -9671,7 +9671,7 @@
       <c r="D95" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F95" s="2" t="s">
@@ -9683,10 +9683,10 @@
       <c r="H95" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I95" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J95" s="3" t="s">
+      <c r="I95" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J95" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9695,7 +9695,7 @@
         <v>176</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>18</v>
@@ -9727,7 +9727,7 @@
         <v>177</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>18</v>
@@ -9744,7 +9744,7 @@
       <c r="G97" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H97" s="2" t="s">
+      <c r="H97" s="3" t="s">
         <v>74</v>
       </c>
       <c r="I97" s="2" t="s">
@@ -9764,16 +9764,16 @@
       <c r="C98" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D98" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E98" s="3" t="s">
+      <c r="D98" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G98" s="3" t="s">
+      <c r="G98" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H98" s="2" t="s">
@@ -9791,7 +9791,7 @@
         <v>179</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>17</v>
@@ -9802,7 +9802,7 @@
       <c r="E99" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F99" s="3" t="s">
+      <c r="F99" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G99" s="2" t="s">
@@ -9814,7 +9814,7 @@
       <c r="I99" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J99" s="3" t="s">
+      <c r="J99" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9831,7 +9831,7 @@
       <c r="D100" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E100" s="2" t="s">
+      <c r="E100" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F100" s="2" t="s">
@@ -9887,7 +9887,7 @@
         <v>182</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C102" s="2" t="s">
         <v>18</v>
@@ -9910,7 +9910,7 @@
       <c r="I102" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J102" s="2" t="s">
+      <c r="J102" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -9919,7 +9919,7 @@
         <v>183</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C103" s="2" t="s">
         <v>17</v>
@@ -9965,10 +9965,10 @@
       <c r="F104" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G104" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H104" s="3" t="s">
+      <c r="G104" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H104" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I104" s="2" t="s">
@@ -9983,7 +9983,7 @@
         <v>185</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>18</v>
@@ -10058,7 +10058,7 @@
       <c r="E107" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F107" s="2" t="s">
+      <c r="F107" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G107" s="2" t="s">
@@ -10099,7 +10099,7 @@
       <c r="H108" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I108" s="2" t="s">
+      <c r="I108" s="3" t="s">
         <v>74</v>
       </c>
       <c r="J108" s="2" t="s">
@@ -10143,7 +10143,7 @@
         <v>190</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>18</v>
@@ -10175,12 +10175,12 @@
         <v>191</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D111" s="3" t="s">
+      <c r="D111" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E111" s="2" t="s">
@@ -10195,7 +10195,7 @@
       <c r="H111" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I111" s="3" t="s">
+      <c r="I111" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J111" s="2" t="s">
@@ -10207,7 +10207,7 @@
         <v>192</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C112" s="2" t="s">
         <v>18</v>
@@ -10215,13 +10215,13 @@
       <c r="D112" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E112" s="3" t="s">
+      <c r="E112" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G112" s="3" t="s">
+      <c r="G112" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H112" s="2" t="s">
@@ -10244,7 +10244,7 @@
       <c r="C113" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D113" s="2" t="s">
+      <c r="D113" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E113" s="2" t="s">
@@ -10256,7 +10256,7 @@
       <c r="G113" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H113" s="2" t="s">
+      <c r="H113" s="3" t="s">
         <v>74</v>
       </c>
       <c r="I113" s="2" t="s">
@@ -10335,7 +10335,7 @@
         <v>196</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>18</v>
@@ -10404,22 +10404,22 @@
       <c r="C118" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D118" s="3" t="s">
+      <c r="D118" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F118" s="3" t="s">
+      <c r="F118" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H118" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I118" s="3" t="s">
+      <c r="H118" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I118" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J118" s="2" t="s">
@@ -10431,7 +10431,7 @@
         <v>199</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C119" s="2" t="s">
         <v>17</v>
@@ -10495,12 +10495,12 @@
         <v>201</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D121" s="3" t="s">
+      <c r="D121" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E121" s="2" t="s">
@@ -10518,7 +10518,7 @@
       <c r="I121" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J121" s="3" t="s">
+      <c r="J121" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -10559,7 +10559,7 @@
         <v>203</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C123" s="2" t="s">
         <v>17</v>
@@ -10591,7 +10591,7 @@
         <v>204</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>17</v>
@@ -10695,19 +10695,19 @@
       <c r="D127" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E127" s="3" t="s">
+      <c r="E127" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F127" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G127" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H127" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I127" s="3" t="s">
+      <c r="G127" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I127" s="2" t="s">
         <v>74</v>
       </c>
       <c r="J127" s="2" t="s">
@@ -10719,7 +10719,7 @@
         <v>208</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C128" s="2" t="s">
         <v>17</v>
@@ -10783,7 +10783,7 @@
         <v>210</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>18</v>
@@ -10797,7 +10797,7 @@
       <c r="F130" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G130" s="2" t="s">
+      <c r="G130" s="3" t="s">
         <v>74</v>
       </c>
       <c r="H130" s="2" t="s">
@@ -10815,7 +10815,7 @@
         <v>211</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C131" s="2" t="s">
         <v>18</v>
@@ -10826,7 +10826,7 @@
       <c r="E131" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F131" s="3" t="s">
+      <c r="F131" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G131" s="2" t="s">
@@ -10835,10 +10835,10 @@
       <c r="H131" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I131" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="J131" s="3" t="s">
+      <c r="I131" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J131" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -10847,7 +10847,7 @@
         <v>212</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>18</v>
@@ -10855,7 +10855,7 @@
       <c r="D132" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E132" s="2" t="s">
+      <c r="E132" s="3" t="s">
         <v>74</v>
       </c>
       <c r="F132" s="2" t="s">
@@ -10879,7 +10879,7 @@
         <v>213</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>17</v>
@@ -10948,10 +10948,10 @@
       <c r="C135" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D135" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E135" s="3" t="s">
+      <c r="D135" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E135" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F135" s="2" t="s">
@@ -10963,10 +10963,10 @@
       <c r="H135" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I135" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J135" s="3" t="s">
+      <c r="I135" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J135" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -10989,10 +10989,10 @@
       <c r="F136" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G136" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H136" s="3" t="s">
+      <c r="G136" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H136" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I136" s="2" t="s">
@@ -11088,7 +11088,7 @@
       <c r="G139" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H139" s="2" t="s">
+      <c r="H139" s="3" t="s">
         <v>74</v>
       </c>
       <c r="I139" s="2" t="s">
@@ -11103,18 +11103,18 @@
         <v>220</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D140" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E140" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F140" s="3" t="s">
+      <c r="D140" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F140" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G140" s="2" t="s">
@@ -11146,7 +11146,7 @@
       <c r="E141" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F141" s="2" t="s">
+      <c r="F141" s="3" t="s">
         <v>74</v>
       </c>
       <c r="G141" s="2" t="s">
@@ -11172,7 +11172,7 @@
       <c r="C142" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D142" s="3" t="s">
+      <c r="D142" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E142" s="2" t="s">
@@ -11181,7 +11181,7 @@
       <c r="F142" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G142" s="3" t="s">
+      <c r="G142" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H142" s="2" t="s">
@@ -11263,7 +11263,7 @@
         <v>225</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>18</v>
@@ -11318,7 +11318,7 @@
       <c r="I146" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J146" s="2" t="s">
+      <c r="J146" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -11327,7 +11327,7 @@
         <v>227</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>18</v>
@@ -11359,7 +11359,7 @@
         <v>228</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>17</v>
@@ -11391,30 +11391,30 @@
         <v>229</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D149" s="3" t="s">
+      <c r="D149" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F149" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G149" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="H149" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I149" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J149" s="3" t="s">
+      <c r="F149" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I149" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J149" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -16415,7 +16415,7 @@
         <v>92</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -16487,7 +16487,7 @@
         <v>101</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
@@ -16503,7 +16503,7 @@
         <v>103</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -16535,7 +16535,7 @@
         <v>107</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
@@ -16543,7 +16543,7 @@
         <v>108</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29">
@@ -16575,7 +16575,7 @@
         <v>112</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
@@ -16583,7 +16583,7 @@
         <v>113</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
@@ -16591,7 +16591,7 @@
         <v>114</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35">
@@ -16607,7 +16607,7 @@
         <v>116</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37">
@@ -16631,7 +16631,7 @@
         <v>119</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40">
@@ -16639,7 +16639,7 @@
         <v>120</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41">
@@ -16647,7 +16647,7 @@
         <v>121</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42">
@@ -16663,7 +16663,7 @@
         <v>123</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
@@ -16671,7 +16671,7 @@
         <v>124</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45">
@@ -16679,7 +16679,7 @@
         <v>125</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46">
@@ -16687,7 +16687,7 @@
         <v>126</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47">
@@ -16695,7 +16695,7 @@
         <v>127</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
@@ -16703,7 +16703,7 @@
         <v>128</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49">
@@ -16711,7 +16711,7 @@
         <v>129</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
@@ -16719,7 +16719,7 @@
         <v>130</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51">
@@ -16735,7 +16735,7 @@
         <v>132</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="53">
@@ -16751,7 +16751,7 @@
         <v>134</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55">
@@ -16775,7 +16775,7 @@
         <v>137</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58">
@@ -16791,7 +16791,7 @@
         <v>139</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60">
@@ -16799,7 +16799,7 @@
         <v>140</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="61">
@@ -16815,7 +16815,7 @@
         <v>142</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63">
@@ -16823,7 +16823,7 @@
         <v>143</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="64">
@@ -16847,7 +16847,7 @@
         <v>146</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="67">
@@ -16863,7 +16863,7 @@
         <v>148</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69">
@@ -16879,7 +16879,7 @@
         <v>150</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="71">
@@ -16895,7 +16895,7 @@
         <v>152</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="73">
@@ -16903,7 +16903,7 @@
         <v>153</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74">
@@ -16927,7 +16927,7 @@
         <v>156</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="77">
@@ -16935,7 +16935,7 @@
         <v>157</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="78">
@@ -16943,7 +16943,7 @@
         <v>158</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="79">
@@ -16951,7 +16951,7 @@
         <v>159</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80">
@@ -16959,7 +16959,7 @@
         <v>160</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="81">
@@ -16967,7 +16967,7 @@
         <v>161</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="82">
@@ -16975,7 +16975,7 @@
         <v>162</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="83">
@@ -16983,7 +16983,7 @@
         <v>163</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="84">
@@ -16991,7 +16991,7 @@
         <v>164</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="85">
@@ -16999,7 +16999,7 @@
         <v>165</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86">
@@ -17039,7 +17039,7 @@
         <v>170</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91">
@@ -17055,7 +17055,7 @@
         <v>172</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="93">
@@ -17079,7 +17079,7 @@
         <v>175</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="96">
@@ -17087,7 +17087,7 @@
         <v>176</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97">
@@ -17095,7 +17095,7 @@
         <v>177</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="98">
@@ -17111,7 +17111,7 @@
         <v>179</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="100">
@@ -17135,7 +17135,7 @@
         <v>182</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="103">
@@ -17143,7 +17143,7 @@
         <v>183</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="104">
@@ -17159,7 +17159,7 @@
         <v>185</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="106">
@@ -17199,7 +17199,7 @@
         <v>190</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="111">
@@ -17207,7 +17207,7 @@
         <v>191</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="112">
@@ -17215,7 +17215,7 @@
         <v>192</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="113">
@@ -17247,7 +17247,7 @@
         <v>196</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="117">
@@ -17271,7 +17271,7 @@
         <v>199</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="120">
@@ -17287,7 +17287,7 @@
         <v>201</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122">
@@ -17303,7 +17303,7 @@
         <v>203</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124">
@@ -17311,7 +17311,7 @@
         <v>204</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125">
@@ -17343,7 +17343,7 @@
         <v>208</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="129">
@@ -17359,7 +17359,7 @@
         <v>210</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="131">
@@ -17367,7 +17367,7 @@
         <v>211</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="132">
@@ -17375,7 +17375,7 @@
         <v>212</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133">
@@ -17383,7 +17383,7 @@
         <v>213</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="134">
@@ -17439,7 +17439,7 @@
         <v>220</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="141">
@@ -17479,7 +17479,7 @@
         <v>225</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="146">
@@ -17495,7 +17495,7 @@
         <v>227</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="148">
@@ -17503,7 +17503,7 @@
         <v>228</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="149">
@@ -17511,7 +17511,7 @@
         <v>229</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="150">

</xml_diff>